<commit_message>
feat(combat): accelerate hook flight and retrieval by fifty percent
</commit_message>
<xml_diff>
--- a/GameData/GameData_Skill.xlsx
+++ b/GameData/GameData_Skill.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillDefinition" sheetId="1" r:id="R176e71136aeb48d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillParameter" sheetId="2" r:id="R273319158eb34368"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillDefinition" sheetId="1" r:id="Rb912bf6d62f8484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillParameter" sheetId="2" r:id="R9ce78df218554572"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1924,7 +1924,7 @@
         <x:v>ProjectileSpeed</x:v>
       </x:c>
       <x:c r="C54" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D54" s="4" t="str">
         <x:v>사용자 지정; 미지정 값은 초기 밸런스</x:v>
@@ -1938,7 +1938,7 @@
         <x:v>PullSpeed</x:v>
       </x:c>
       <x:c r="C55" s="14" t="n">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
         <x:v>사용자 지정; 미지정 값은 초기 밸런스</x:v>
@@ -2596,7 +2596,7 @@
         <x:v>RetrieveSeconds</x:v>
       </x:c>
       <x:c r="C102" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>2026-10-04 스킬 조작·연출 개선</x:v>

</xml_diff>